<commit_message>
feat(mlg): depurar XLSX — eliminar productos fuera de categoría
Eliminados 28 filas (9 tipos + sus variantes de color) que no pertenecen
a las categorías MLG: bicchieri, coppette, brocche e bottiglie, piati,
alzate, olio e pepe, portaghiaccio, portaposate.

Tipos eliminados de Complementos:
- Bol para Mascotas (Kane) — 4 SKUs
- Pantalla de Lámpara (Andalusia, Calypso, Cleopatra, Joshua) — 8 SKUs
- Base de Lámpara (Calypso, Joshua) — 2 SKUs
- Base Piña Serena (Serena) — 5 SKUs
- Base Piña (Melissa) — 4 SKUs

SKUs: 430 → 402 | Resumen por Familia actualizado.

https://claude.ai/code/session_011RLxBSyYr3jWuDg26Bu8wU
</commit_message>
<xml_diff>
--- a/MLG_catalog_data.xlsx
+++ b/MLG_catalog_data.xlsx
@@ -585,7 +585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H431"/>
+  <dimension ref="A1:H403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10402,12 +10402,12 @@
       </c>
       <c r="B379" s="14" t="inlineStr">
         <is>
-          <t>Kane</t>
+          <t>Antartica</t>
         </is>
       </c>
       <c r="C379" s="14" t="inlineStr">
         <is>
-          <t>Bol para Mascotas</t>
+          <t>Cubitera</t>
         </is>
       </c>
       <c r="D379" s="14" t="inlineStr">
@@ -10422,17 +10422,17 @@
       </c>
       <c r="F379" s="14" t="inlineStr">
         <is>
-          <t>H.KAN1</t>
+          <t>H.PBO18</t>
         </is>
       </c>
       <c r="G379" s="14" t="inlineStr">
         <is>
-          <t>Rojo</t>
+          <t>Ámbar</t>
         </is>
       </c>
       <c r="H379" s="15" t="inlineStr">
         <is>
-          <t>$325.000</t>
+          <t>$636.000</t>
         </is>
       </c>
     </row>
@@ -10444,17 +10444,17 @@
       <c r="E380" s="4" t="inlineStr"/>
       <c r="F380" s="4" t="inlineStr">
         <is>
-          <t>H.KAN2</t>
+          <t>H.PBO19</t>
         </is>
       </c>
       <c r="G380" s="4" t="inlineStr">
         <is>
-          <t>Ámbar</t>
+          <t>Azul</t>
         </is>
       </c>
       <c r="H380" s="5" t="inlineStr">
         <is>
-          <t>$325.000</t>
+          <t>$636.000</t>
         </is>
       </c>
     </row>
@@ -10466,17 +10466,17 @@
       <c r="E381" s="14" t="inlineStr"/>
       <c r="F381" s="14" t="inlineStr">
         <is>
-          <t>H.KAN3</t>
+          <t>H.PBO20</t>
         </is>
       </c>
       <c r="G381" s="14" t="inlineStr">
         <is>
-          <t>Azul Real</t>
+          <t>Transparente</t>
         </is>
       </c>
       <c r="H381" s="15" t="inlineStr">
         <is>
-          <t>$325.000</t>
+          <t>$636.000</t>
         </is>
       </c>
     </row>
@@ -10488,7 +10488,7 @@
       <c r="E382" s="4" t="inlineStr"/>
       <c r="F382" s="4" t="inlineStr">
         <is>
-          <t>H.KAN4</t>
+          <t>H.PBO21</t>
         </is>
       </c>
       <c r="G382" s="4" t="inlineStr">
@@ -10498,49 +10498,29 @@
       </c>
       <c r="H382" s="5" t="inlineStr">
         <is>
-          <t>$325.000</t>
+          <t>$636.000</t>
         </is>
       </c>
     </row>
     <row r="383" ht="16" customHeight="1">
-      <c r="A383" s="14" t="inlineStr">
-        <is>
-          <t>Complementos</t>
-        </is>
-      </c>
-      <c r="B383" s="14" t="inlineStr">
-        <is>
-          <t>Andalusia</t>
-        </is>
-      </c>
-      <c r="C383" s="14" t="inlineStr">
-        <is>
-          <t>Pantalla de Lámpara</t>
-        </is>
-      </c>
-      <c r="D383" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E383" s="14" t="inlineStr">
-        <is>
-          <t>Acrílico</t>
-        </is>
-      </c>
+      <c r="A383" s="14" t="inlineStr"/>
+      <c r="B383" s="14" t="inlineStr"/>
+      <c r="C383" s="14" t="inlineStr"/>
+      <c r="D383" s="14" t="inlineStr"/>
+      <c r="E383" s="14" t="inlineStr"/>
       <c r="F383" s="14" t="inlineStr">
         <is>
-          <t>H.LAM.AND1</t>
+          <t>H.PBO22</t>
         </is>
       </c>
       <c r="G383" s="14" t="inlineStr">
         <is>
-          <t>Transparente</t>
+          <t>Rojo</t>
         </is>
       </c>
       <c r="H383" s="15" t="inlineStr">
         <is>
-          <t>$269.000</t>
+          <t>$636.000</t>
         </is>
       </c>
     </row>
@@ -10552,17 +10532,17 @@
       <c r="E384" s="4" t="inlineStr"/>
       <c r="F384" s="4" t="inlineStr">
         <is>
-          <t>H.LAM.AND2</t>
+          <t>H.PBO29</t>
         </is>
       </c>
       <c r="G384" s="4" t="inlineStr">
         <is>
-          <t>Rojo</t>
+          <t>Blanco Esmerilado</t>
         </is>
       </c>
       <c r="H384" s="5" t="inlineStr">
         <is>
-          <t>$269.000</t>
+          <t>$665.000</t>
         </is>
       </c>
     </row>
@@ -10574,423 +10554,363 @@
       <c r="E385" s="14" t="inlineStr"/>
       <c r="F385" s="14" t="inlineStr">
         <is>
-          <t>H.LAM.AND3</t>
+          <t>H.PBO32</t>
         </is>
       </c>
       <c r="G385" s="14" t="inlineStr">
         <is>
+          <t>Rojo Esmerilado</t>
+        </is>
+      </c>
+      <c r="H385" s="15" t="inlineStr">
+        <is>
+          <t>$665.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="386" ht="16" customHeight="1">
+      <c r="A386" s="4" t="inlineStr"/>
+      <c r="B386" s="4" t="inlineStr"/>
+      <c r="C386" s="4" t="inlineStr"/>
+      <c r="D386" s="4" t="inlineStr"/>
+      <c r="E386" s="4" t="inlineStr"/>
+      <c r="F386" s="4" t="inlineStr">
+        <is>
+          <t>H.PBO35</t>
+        </is>
+      </c>
+      <c r="G386" s="4" t="inlineStr">
+        <is>
+          <t>Azul Esmerilado</t>
+        </is>
+      </c>
+      <c r="H386" s="5" t="inlineStr">
+        <is>
+          <t>$665.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="387" ht="16" customHeight="1">
+      <c r="A387" s="14" t="inlineStr"/>
+      <c r="B387" s="14" t="inlineStr"/>
+      <c r="C387" s="14" t="inlineStr"/>
+      <c r="D387" s="14" t="inlineStr"/>
+      <c r="E387" s="14" t="inlineStr"/>
+      <c r="F387" s="14" t="inlineStr">
+        <is>
+          <t>H.PBO37</t>
+        </is>
+      </c>
+      <c r="G387" s="14" t="inlineStr">
+        <is>
+          <t>Dorado</t>
+        </is>
+      </c>
+      <c r="H387" s="15" t="inlineStr">
+        <is>
+          <t>$794.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="388" ht="16" customHeight="1">
+      <c r="A388" s="14" t="inlineStr">
+        <is>
+          <t>Complementos</t>
+        </is>
+      </c>
+      <c r="B388" s="14" t="inlineStr">
+        <is>
+          <t>Filippo</t>
+        </is>
+      </c>
+      <c r="C388" s="14" t="inlineStr">
+        <is>
+          <t>Soportaborellas</t>
+        </is>
+      </c>
+      <c r="D388" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E388" s="14" t="inlineStr">
+        <is>
+          <t>Acrílico</t>
+        </is>
+      </c>
+      <c r="F388" s="14" t="inlineStr">
+        <is>
+          <t>H.PBO24</t>
+        </is>
+      </c>
+      <c r="G388" s="14" t="inlineStr">
+        <is>
+          <t>Transparente</t>
+        </is>
+      </c>
+      <c r="H388" s="15" t="inlineStr">
+        <is>
+          <t>$414.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="389" ht="16" customHeight="1">
+      <c r="A389" s="4" t="inlineStr"/>
+      <c r="B389" s="4" t="inlineStr"/>
+      <c r="C389" s="4" t="inlineStr"/>
+      <c r="D389" s="4" t="inlineStr"/>
+      <c r="E389" s="4" t="inlineStr"/>
+      <c r="F389" s="4" t="inlineStr">
+        <is>
+          <t>H.PBO26</t>
+        </is>
+      </c>
+      <c r="G389" s="4" t="inlineStr">
+        <is>
+          <t>Rojo</t>
+        </is>
+      </c>
+      <c r="H389" s="5" t="inlineStr">
+        <is>
+          <t>$414.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="390" ht="16" customHeight="1">
+      <c r="A390" s="14" t="inlineStr"/>
+      <c r="B390" s="14" t="inlineStr"/>
+      <c r="C390" s="14" t="inlineStr"/>
+      <c r="D390" s="14" t="inlineStr"/>
+      <c r="E390" s="14" t="inlineStr"/>
+      <c r="F390" s="14" t="inlineStr">
+        <is>
+          <t>H.PBO30</t>
+        </is>
+      </c>
+      <c r="G390" s="14" t="inlineStr">
+        <is>
+          <t>Turquesa</t>
+        </is>
+      </c>
+      <c r="H390" s="15" t="inlineStr">
+        <is>
+          <t>$414.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="391" ht="16" customHeight="1">
+      <c r="A391" s="14" t="inlineStr">
+        <is>
+          <t>Complementos</t>
+        </is>
+      </c>
+      <c r="B391" s="14" t="inlineStr">
+        <is>
+          <t>Bonnie &amp; Clyde</t>
+        </is>
+      </c>
+      <c r="C391" s="14" t="inlineStr">
+        <is>
+          <t>Sal y Pimienta</t>
+        </is>
+      </c>
+      <c r="D391" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E391" s="14" t="inlineStr">
+        <is>
+          <t>Acrílico</t>
+        </is>
+      </c>
+      <c r="F391" s="14" t="inlineStr">
+        <is>
+          <t>H.SAL.BEC1</t>
+        </is>
+      </c>
+      <c r="G391" s="14" t="inlineStr">
+        <is>
           <t>Verde</t>
         </is>
       </c>
-      <c r="H385" s="15" t="inlineStr">
-        <is>
-          <t>$269.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="386" ht="16" customHeight="1">
-      <c r="A386" s="14" t="inlineStr">
+      <c r="H391" s="15" t="inlineStr">
+        <is>
+          <t>$222.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="392" ht="16" customHeight="1">
+      <c r="A392" s="4" t="inlineStr"/>
+      <c r="B392" s="4" t="inlineStr"/>
+      <c r="C392" s="4" t="inlineStr"/>
+      <c r="D392" s="4" t="inlineStr"/>
+      <c r="E392" s="4" t="inlineStr"/>
+      <c r="F392" s="4" t="inlineStr">
+        <is>
+          <t>H.SAL.BEC2</t>
+        </is>
+      </c>
+      <c r="G392" s="4" t="inlineStr">
+        <is>
+          <t>Transparente</t>
+        </is>
+      </c>
+      <c r="H392" s="5" t="inlineStr">
+        <is>
+          <t>$222.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="393" ht="16" customHeight="1">
+      <c r="A393" s="14" t="inlineStr"/>
+      <c r="B393" s="14" t="inlineStr"/>
+      <c r="C393" s="14" t="inlineStr"/>
+      <c r="D393" s="14" t="inlineStr"/>
+      <c r="E393" s="14" t="inlineStr"/>
+      <c r="F393" s="14" t="inlineStr">
+        <is>
+          <t>H.SAL.BEC3</t>
+        </is>
+      </c>
+      <c r="G393" s="14" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="H393" s="15" t="inlineStr">
+        <is>
+          <t>$222.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="394" ht="16" customHeight="1">
+      <c r="A394" s="4" t="inlineStr"/>
+      <c r="B394" s="4" t="inlineStr"/>
+      <c r="C394" s="4" t="inlineStr"/>
+      <c r="D394" s="4" t="inlineStr"/>
+      <c r="E394" s="4" t="inlineStr"/>
+      <c r="F394" s="4" t="inlineStr">
+        <is>
+          <t>H.SAL.BEC5</t>
+        </is>
+      </c>
+      <c r="G394" s="4" t="inlineStr">
+        <is>
+          <t>Rojo</t>
+        </is>
+      </c>
+      <c r="H394" s="5" t="inlineStr">
+        <is>
+          <t>$222.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="395" ht="16" customHeight="1">
+      <c r="A395" s="14" t="inlineStr"/>
+      <c r="B395" s="14" t="inlineStr"/>
+      <c r="C395" s="14" t="inlineStr"/>
+      <c r="D395" s="14" t="inlineStr"/>
+      <c r="E395" s="14" t="inlineStr"/>
+      <c r="F395" s="14" t="inlineStr">
+        <is>
+          <t>H.SAL.BEC6</t>
+        </is>
+      </c>
+      <c r="G395" s="14" t="inlineStr">
+        <is>
+          <t>Dorado</t>
+        </is>
+      </c>
+      <c r="H395" s="15" t="inlineStr">
+        <is>
+          <t>$222.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="396" ht="16" customHeight="1">
+      <c r="A396" s="14" t="inlineStr">
         <is>
           <t>Complementos</t>
         </is>
       </c>
-      <c r="B386" s="14" t="inlineStr">
-        <is>
-          <t>Calypso</t>
-        </is>
-      </c>
-      <c r="C386" s="14" t="inlineStr">
-        <is>
-          <t>Pantalla de Lámpara</t>
-        </is>
-      </c>
-      <c r="D386" s="14" t="inlineStr">
+      <c r="B396" s="14" t="inlineStr">
+        <is>
+          <t>Casanova</t>
+        </is>
+      </c>
+      <c r="C396" s="14" t="inlineStr">
+        <is>
+          <t>Salero</t>
+        </is>
+      </c>
+      <c r="D396" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E386" s="14" t="inlineStr">
+      <c r="E396" s="14" t="inlineStr">
         <is>
           <t>Acrílico</t>
         </is>
       </c>
-      <c r="F386" s="14" t="inlineStr">
-        <is>
-          <t>H.LAM.CAL11</t>
-        </is>
-      </c>
-      <c r="G386" s="14" t="inlineStr">
-        <is>
-          <t>Gris</t>
-        </is>
-      </c>
-      <c r="H386" s="15" t="inlineStr">
-        <is>
-          <t>$611.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="387" ht="16" customHeight="1">
-      <c r="A387" s="4" t="inlineStr"/>
-      <c r="B387" s="4" t="inlineStr"/>
-      <c r="C387" s="4" t="inlineStr"/>
-      <c r="D387" s="4" t="inlineStr"/>
-      <c r="E387" s="4" t="inlineStr"/>
-      <c r="F387" s="4" t="inlineStr">
-        <is>
-          <t>H.LAM.CAL8</t>
-        </is>
-      </c>
-      <c r="G387" s="4" t="inlineStr">
+      <c r="F396" s="14" t="inlineStr">
+        <is>
+          <t>H.SAL.CAS1</t>
+        </is>
+      </c>
+      <c r="G396" s="14" t="inlineStr">
         <is>
           <t>Transparente</t>
         </is>
       </c>
-      <c r="H387" s="5" t="inlineStr">
-        <is>
-          <t>$611.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="388" ht="16" customHeight="1">
-      <c r="A388" s="14" t="inlineStr"/>
-      <c r="B388" s="14" t="inlineStr"/>
-      <c r="C388" s="14" t="inlineStr"/>
-      <c r="D388" s="14" t="inlineStr"/>
-      <c r="E388" s="14" t="inlineStr"/>
-      <c r="F388" s="14" t="inlineStr">
-        <is>
-          <t>H.LAM.CAL9</t>
-        </is>
-      </c>
-      <c r="G388" s="14" t="inlineStr">
-        <is>
-          <t>Dorado</t>
-        </is>
-      </c>
-      <c r="H388" s="15" t="inlineStr">
-        <is>
-          <t>$611.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="389" ht="16" customHeight="1">
-      <c r="A389" s="14" t="inlineStr">
-        <is>
-          <t>Complementos</t>
-        </is>
-      </c>
-      <c r="B389" s="14" t="inlineStr">
-        <is>
-          <t>Calypso</t>
-        </is>
-      </c>
-      <c r="C389" s="14" t="inlineStr">
-        <is>
-          <t>Base de Lámpara</t>
-        </is>
-      </c>
-      <c r="D389" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E389" s="14" t="inlineStr">
-        <is>
-          <t>Acrílico</t>
-        </is>
-      </c>
-      <c r="F389" s="14" t="inlineStr">
-        <is>
-          <t>H.LAM.CAL6</t>
-        </is>
-      </c>
-      <c r="G389" s="14" t="inlineStr">
-        <is>
-          <t>Transparente</t>
-        </is>
-      </c>
-      <c r="H389" s="15" t="inlineStr">
-        <is>
-          <t>$1.459.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="390" ht="16" customHeight="1">
-      <c r="A390" s="14" t="inlineStr">
-        <is>
-          <t>Complementos</t>
-        </is>
-      </c>
-      <c r="B390" s="14" t="inlineStr">
-        <is>
-          <t>Cleopatra</t>
-        </is>
-      </c>
-      <c r="C390" s="14" t="inlineStr">
-        <is>
-          <t>Pantalla de Lámpara</t>
-        </is>
-      </c>
-      <c r="D390" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E390" s="14" t="inlineStr">
-        <is>
-          <t>Acrílico</t>
-        </is>
-      </c>
-      <c r="F390" s="14" t="inlineStr">
-        <is>
-          <t>H.LAM.CLE5</t>
-        </is>
-      </c>
-      <c r="G390" s="14" t="inlineStr">
-        <is>
-          <t>Transparente</t>
-        </is>
-      </c>
-      <c r="H390" s="15" t="inlineStr">
-        <is>
-          <t>$269.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="391" ht="16" customHeight="1">
-      <c r="A391" s="4" t="inlineStr"/>
-      <c r="B391" s="4" t="inlineStr"/>
-      <c r="C391" s="4" t="inlineStr"/>
-      <c r="D391" s="4" t="inlineStr"/>
-      <c r="E391" s="4" t="inlineStr"/>
-      <c r="F391" s="4" t="inlineStr">
-        <is>
-          <t>H.LAM.CLE6</t>
-        </is>
-      </c>
-      <c r="G391" s="4" t="inlineStr">
-        <is>
-          <t>Naranja</t>
-        </is>
-      </c>
-      <c r="H391" s="5" t="inlineStr">
-        <is>
-          <t>$269.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="392" ht="16" customHeight="1">
-      <c r="A392" s="14" t="inlineStr"/>
-      <c r="B392" s="14" t="inlineStr"/>
-      <c r="C392" s="14" t="inlineStr"/>
-      <c r="D392" s="14" t="inlineStr"/>
-      <c r="E392" s="14" t="inlineStr"/>
-      <c r="F392" s="14" t="inlineStr">
-        <is>
-          <t>H.LAM.CLE7</t>
-        </is>
-      </c>
-      <c r="G392" s="14" t="inlineStr">
-        <is>
-          <t>Rojo</t>
-        </is>
-      </c>
-      <c r="H392" s="15" t="inlineStr">
-        <is>
-          <t>$269.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="393" ht="16" customHeight="1">
-      <c r="A393" s="4" t="inlineStr"/>
-      <c r="B393" s="4" t="inlineStr"/>
-      <c r="C393" s="4" t="inlineStr"/>
-      <c r="D393" s="4" t="inlineStr"/>
-      <c r="E393" s="4" t="inlineStr"/>
-      <c r="F393" s="4" t="inlineStr">
-        <is>
-          <t>H.LAM.CLE8</t>
-        </is>
-      </c>
-      <c r="G393" s="4" t="inlineStr">
-        <is>
-          <t>Turquesa</t>
-        </is>
-      </c>
-      <c r="H393" s="5" t="inlineStr">
-        <is>
-          <t>$269.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="394" ht="16" customHeight="1">
-      <c r="A394" s="14" t="inlineStr">
-        <is>
-          <t>Complementos</t>
-        </is>
-      </c>
-      <c r="B394" s="14" t="inlineStr">
-        <is>
-          <t>Joshua</t>
-        </is>
-      </c>
-      <c r="C394" s="14" t="inlineStr">
-        <is>
-          <t>Pantalla de Lámpara</t>
-        </is>
-      </c>
-      <c r="D394" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E394" s="14" t="inlineStr">
-        <is>
-          <t>Acrílico</t>
-        </is>
-      </c>
-      <c r="F394" s="14" t="inlineStr">
-        <is>
-          <t>H.LAM.JOS10</t>
-        </is>
-      </c>
-      <c r="G394" s="14" t="inlineStr">
-        <is>
-          <t>Blanco Opaco</t>
-        </is>
-      </c>
-      <c r="H394" s="15" t="inlineStr">
-        <is>
-          <t>$428.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="395" ht="16" customHeight="1">
-      <c r="A395" s="4" t="inlineStr"/>
-      <c r="B395" s="4" t="inlineStr"/>
-      <c r="C395" s="4" t="inlineStr"/>
-      <c r="D395" s="4" t="inlineStr"/>
-      <c r="E395" s="4" t="inlineStr"/>
-      <c r="F395" s="4" t="inlineStr">
-        <is>
-          <t>H.LAM.JOS7</t>
-        </is>
-      </c>
-      <c r="G395" s="4" t="inlineStr">
-        <is>
-          <t>Transparente</t>
-        </is>
-      </c>
-      <c r="H395" s="5" t="inlineStr">
-        <is>
-          <t>$428.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="396" ht="16" customHeight="1">
-      <c r="A396" s="14" t="inlineStr"/>
-      <c r="B396" s="14" t="inlineStr"/>
-      <c r="C396" s="14" t="inlineStr"/>
-      <c r="D396" s="14" t="inlineStr"/>
-      <c r="E396" s="14" t="inlineStr"/>
-      <c r="F396" s="14" t="inlineStr">
-        <is>
-          <t>H.LAM.JOS9</t>
-        </is>
-      </c>
-      <c r="G396" s="14" t="inlineStr">
-        <is>
-          <t>Gris Opaco</t>
-        </is>
-      </c>
       <c r="H396" s="15" t="inlineStr">
         <is>
-          <t>$428.000</t>
+          <t>$55.000</t>
         </is>
       </c>
     </row>
     <row r="397" ht="16" customHeight="1">
-      <c r="A397" s="14" t="inlineStr">
-        <is>
-          <t>Complementos</t>
-        </is>
-      </c>
-      <c r="B397" s="14" t="inlineStr">
-        <is>
-          <t>Joshua</t>
-        </is>
-      </c>
-      <c r="C397" s="14" t="inlineStr">
-        <is>
-          <t>Base de Lámpara</t>
-        </is>
-      </c>
-      <c r="D397" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E397" s="14" t="inlineStr">
-        <is>
-          <t>Acrílico</t>
-        </is>
-      </c>
-      <c r="F397" s="14" t="inlineStr">
-        <is>
-          <t>H.LAM.JOS11</t>
-        </is>
-      </c>
-      <c r="G397" s="14" t="inlineStr">
-        <is>
-          <t>Transparente</t>
-        </is>
-      </c>
-      <c r="H397" s="15" t="inlineStr">
-        <is>
-          <t>$755.000</t>
+      <c r="A397" s="4" t="inlineStr"/>
+      <c r="B397" s="4" t="inlineStr"/>
+      <c r="C397" s="4" t="inlineStr"/>
+      <c r="D397" s="4" t="inlineStr"/>
+      <c r="E397" s="4" t="inlineStr"/>
+      <c r="F397" s="4" t="inlineStr">
+        <is>
+          <t>H.SAL.CAS2</t>
+        </is>
+      </c>
+      <c r="G397" s="4" t="inlineStr">
+        <is>
+          <t>Ahumado</t>
+        </is>
+      </c>
+      <c r="H397" s="5" t="inlineStr">
+        <is>
+          <t>$55.000</t>
         </is>
       </c>
     </row>
     <row r="398" ht="16" customHeight="1">
-      <c r="A398" s="14" t="inlineStr">
-        <is>
-          <t>Complementos</t>
-        </is>
-      </c>
-      <c r="B398" s="14" t="inlineStr">
-        <is>
-          <t>Serena</t>
-        </is>
-      </c>
-      <c r="C398" s="14" t="inlineStr">
-        <is>
-          <t>Base Piña Serena</t>
-        </is>
-      </c>
-      <c r="D398" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E398" s="14" t="inlineStr">
-        <is>
-          <t>Acrílico</t>
-        </is>
-      </c>
+      <c r="A398" s="14" t="inlineStr"/>
+      <c r="B398" s="14" t="inlineStr"/>
+      <c r="C398" s="14" t="inlineStr"/>
+      <c r="D398" s="14" t="inlineStr"/>
+      <c r="E398" s="14" t="inlineStr"/>
       <c r="F398" s="14" t="inlineStr">
         <is>
-          <t>H.MAD1</t>
+          <t>H.SAL.CAS3</t>
         </is>
       </c>
       <c r="G398" s="14" t="inlineStr">
         <is>
-          <t>Transparente</t>
+          <t>Verde</t>
         </is>
       </c>
       <c r="H398" s="15" t="inlineStr">
         <is>
-          <t>$550.000</t>
+          <t>$55.000</t>
         </is>
       </c>
     </row>
@@ -11002,39 +10922,59 @@
       <c r="E399" s="4" t="inlineStr"/>
       <c r="F399" s="4" t="inlineStr">
         <is>
-          <t>H.MAD2</t>
+          <t>H.SAL.CAS4</t>
         </is>
       </c>
       <c r="G399" s="4" t="inlineStr">
         <is>
-          <t>Rubí</t>
+          <t>Rojo</t>
         </is>
       </c>
       <c r="H399" s="5" t="inlineStr">
         <is>
-          <t>$550.000</t>
+          <t>$55.000</t>
         </is>
       </c>
     </row>
     <row r="400" ht="16" customHeight="1">
-      <c r="A400" s="14" t="inlineStr"/>
-      <c r="B400" s="14" t="inlineStr"/>
-      <c r="C400" s="14" t="inlineStr"/>
-      <c r="D400" s="14" t="inlineStr"/>
-      <c r="E400" s="14" t="inlineStr"/>
+      <c r="A400" s="14" t="inlineStr">
+        <is>
+          <t>Complementos</t>
+        </is>
+      </c>
+      <c r="B400" s="14" t="inlineStr">
+        <is>
+          <t>Caterina &amp; Vittoria</t>
+        </is>
+      </c>
+      <c r="C400" s="14" t="inlineStr">
+        <is>
+          <t>Sal y Pimienta</t>
+        </is>
+      </c>
+      <c r="D400" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E400" s="14" t="inlineStr">
+        <is>
+          <t>Acrílico</t>
+        </is>
+      </c>
       <c r="F400" s="14" t="inlineStr">
         <is>
-          <t>H.MAD3</t>
+          <t>H.SAL.CEV1</t>
         </is>
       </c>
       <c r="G400" s="14" t="inlineStr">
         <is>
-          <t>Ámbar</t>
+          <t>Transparente</t>
         </is>
       </c>
       <c r="H400" s="15" t="inlineStr">
         <is>
-          <t>$550.000</t>
+          <t>$269.000</t>
         </is>
       </c>
     </row>
@@ -11046,17 +10986,17 @@
       <c r="E401" s="4" t="inlineStr"/>
       <c r="F401" s="4" t="inlineStr">
         <is>
-          <t>H.MAD4</t>
+          <t>H.SAL.CEV2</t>
         </is>
       </c>
       <c r="G401" s="4" t="inlineStr">
         <is>
-          <t>Verde</t>
+          <t>Rubí</t>
         </is>
       </c>
       <c r="H401" s="5" t="inlineStr">
         <is>
-          <t>$550.000</t>
+          <t>$269.000</t>
         </is>
       </c>
     </row>
@@ -11068,778 +11008,70 @@
       <c r="E402" s="14" t="inlineStr"/>
       <c r="F402" s="14" t="inlineStr">
         <is>
-          <t>H.MAD5</t>
+          <t>H.SAL.CEV3</t>
         </is>
       </c>
       <c r="G402" s="14" t="inlineStr">
         <is>
-          <t>Dorado</t>
+          <t>Azul</t>
         </is>
       </c>
       <c r="H402" s="15" t="inlineStr">
         <is>
-          <t>$550.000</t>
+          <t>$269.000</t>
         </is>
       </c>
     </row>
     <row r="403" ht="16" customHeight="1">
-      <c r="A403" s="14" t="inlineStr">
-        <is>
-          <t>Complementos</t>
-        </is>
-      </c>
-      <c r="B403" s="14" t="inlineStr">
-        <is>
-          <t>Melissa</t>
-        </is>
-      </c>
-      <c r="C403" s="14" t="inlineStr">
-        <is>
-          <t>Base Piña</t>
-        </is>
-      </c>
-      <c r="D403" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E403" s="14" t="inlineStr">
-        <is>
-          <t>Acrílico</t>
-        </is>
-      </c>
-      <c r="F403" s="14" t="inlineStr">
-        <is>
-          <t>H.MEL2</t>
-        </is>
-      </c>
-      <c r="G403" s="14" t="inlineStr">
-        <is>
-          <t>Transparente</t>
-        </is>
-      </c>
-      <c r="H403" s="15" t="inlineStr">
-        <is>
-          <t>$1.283.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="404" ht="16" customHeight="1">
-      <c r="A404" s="4" t="inlineStr"/>
-      <c r="B404" s="4" t="inlineStr"/>
-      <c r="C404" s="4" t="inlineStr"/>
-      <c r="D404" s="4" t="inlineStr"/>
-      <c r="E404" s="4" t="inlineStr"/>
-      <c r="F404" s="4" t="inlineStr">
-        <is>
-          <t>H.MEL3</t>
-        </is>
-      </c>
-      <c r="G404" s="4" t="inlineStr">
+      <c r="A403" s="4" t="inlineStr"/>
+      <c r="B403" s="4" t="inlineStr"/>
+      <c r="C403" s="4" t="inlineStr"/>
+      <c r="D403" s="4" t="inlineStr"/>
+      <c r="E403" s="4" t="inlineStr"/>
+      <c r="F403" s="4" t="inlineStr">
+        <is>
+          <t>H.SAL.CEV4</t>
+        </is>
+      </c>
+      <c r="G403" s="4" t="inlineStr">
         <is>
           <t>Verde</t>
         </is>
       </c>
-      <c r="H404" s="5" t="inlineStr">
-        <is>
-          <t>$1.283.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="405" ht="16" customHeight="1">
-      <c r="A405" s="14" t="inlineStr"/>
-      <c r="B405" s="14" t="inlineStr"/>
-      <c r="C405" s="14" t="inlineStr"/>
-      <c r="D405" s="14" t="inlineStr"/>
-      <c r="E405" s="14" t="inlineStr"/>
-      <c r="F405" s="14" t="inlineStr">
-        <is>
-          <t>H.MEL4</t>
-        </is>
-      </c>
-      <c r="G405" s="14" t="inlineStr">
-        <is>
-          <t>Dorado</t>
-        </is>
-      </c>
-      <c r="H405" s="15" t="inlineStr">
-        <is>
-          <t>$1.283.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="406" ht="16" customHeight="1">
-      <c r="A406" s="4" t="inlineStr"/>
-      <c r="B406" s="4" t="inlineStr"/>
-      <c r="C406" s="4" t="inlineStr"/>
-      <c r="D406" s="4" t="inlineStr"/>
-      <c r="E406" s="4" t="inlineStr"/>
-      <c r="F406" s="4" t="inlineStr">
-        <is>
-          <t>H.MEL5</t>
-        </is>
-      </c>
-      <c r="G406" s="4" t="inlineStr">
-        <is>
-          <t>Rubí</t>
-        </is>
-      </c>
-      <c r="H406" s="5" t="inlineStr">
-        <is>
-          <t>$1.283.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="407" ht="16" customHeight="1">
-      <c r="A407" s="14" t="inlineStr">
-        <is>
-          <t>Complementos</t>
-        </is>
-      </c>
-      <c r="B407" s="14" t="inlineStr">
-        <is>
-          <t>Antartica</t>
-        </is>
-      </c>
-      <c r="C407" s="14" t="inlineStr">
-        <is>
-          <t>Cubitera</t>
-        </is>
-      </c>
-      <c r="D407" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E407" s="14" t="inlineStr">
-        <is>
-          <t>Acrílico</t>
-        </is>
-      </c>
-      <c r="F407" s="14" t="inlineStr">
-        <is>
-          <t>H.PBO18</t>
-        </is>
-      </c>
-      <c r="G407" s="14" t="inlineStr">
-        <is>
-          <t>Ámbar</t>
-        </is>
-      </c>
-      <c r="H407" s="15" t="inlineStr">
-        <is>
-          <t>$636.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="408" ht="16" customHeight="1">
-      <c r="A408" s="4" t="inlineStr"/>
-      <c r="B408" s="4" t="inlineStr"/>
-      <c r="C408" s="4" t="inlineStr"/>
-      <c r="D408" s="4" t="inlineStr"/>
-      <c r="E408" s="4" t="inlineStr"/>
-      <c r="F408" s="4" t="inlineStr">
-        <is>
-          <t>H.PBO19</t>
-        </is>
-      </c>
-      <c r="G408" s="4" t="inlineStr">
-        <is>
-          <t>Azul</t>
-        </is>
-      </c>
-      <c r="H408" s="5" t="inlineStr">
-        <is>
-          <t>$636.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="409" ht="16" customHeight="1">
-      <c r="A409" s="14" t="inlineStr"/>
-      <c r="B409" s="14" t="inlineStr"/>
-      <c r="C409" s="14" t="inlineStr"/>
-      <c r="D409" s="14" t="inlineStr"/>
-      <c r="E409" s="14" t="inlineStr"/>
-      <c r="F409" s="14" t="inlineStr">
-        <is>
-          <t>H.PBO20</t>
-        </is>
-      </c>
-      <c r="G409" s="14" t="inlineStr">
-        <is>
-          <t>Transparente</t>
-        </is>
-      </c>
-      <c r="H409" s="15" t="inlineStr">
-        <is>
-          <t>$636.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="410" ht="16" customHeight="1">
-      <c r="A410" s="4" t="inlineStr"/>
-      <c r="B410" s="4" t="inlineStr"/>
-      <c r="C410" s="4" t="inlineStr"/>
-      <c r="D410" s="4" t="inlineStr"/>
-      <c r="E410" s="4" t="inlineStr"/>
-      <c r="F410" s="4" t="inlineStr">
-        <is>
-          <t>H.PBO21</t>
-        </is>
-      </c>
-      <c r="G410" s="4" t="inlineStr">
-        <is>
-          <t>Verde</t>
-        </is>
-      </c>
-      <c r="H410" s="5" t="inlineStr">
-        <is>
-          <t>$636.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="411" ht="16" customHeight="1">
-      <c r="A411" s="14" t="inlineStr"/>
-      <c r="B411" s="14" t="inlineStr"/>
-      <c r="C411" s="14" t="inlineStr"/>
-      <c r="D411" s="14" t="inlineStr"/>
-      <c r="E411" s="14" t="inlineStr"/>
-      <c r="F411" s="14" t="inlineStr">
-        <is>
-          <t>H.PBO22</t>
-        </is>
-      </c>
-      <c r="G411" s="14" t="inlineStr">
-        <is>
-          <t>Rojo</t>
-        </is>
-      </c>
-      <c r="H411" s="15" t="inlineStr">
-        <is>
-          <t>$636.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="412" ht="16" customHeight="1">
-      <c r="A412" s="4" t="inlineStr"/>
-      <c r="B412" s="4" t="inlineStr"/>
-      <c r="C412" s="4" t="inlineStr"/>
-      <c r="D412" s="4" t="inlineStr"/>
-      <c r="E412" s="4" t="inlineStr"/>
-      <c r="F412" s="4" t="inlineStr">
-        <is>
-          <t>H.PBO29</t>
-        </is>
-      </c>
-      <c r="G412" s="4" t="inlineStr">
-        <is>
-          <t>Blanco Esmerilado</t>
-        </is>
-      </c>
-      <c r="H412" s="5" t="inlineStr">
-        <is>
-          <t>$665.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="413" ht="16" customHeight="1">
-      <c r="A413" s="14" t="inlineStr"/>
-      <c r="B413" s="14" t="inlineStr"/>
-      <c r="C413" s="14" t="inlineStr"/>
-      <c r="D413" s="14" t="inlineStr"/>
-      <c r="E413" s="14" t="inlineStr"/>
-      <c r="F413" s="14" t="inlineStr">
-        <is>
-          <t>H.PBO32</t>
-        </is>
-      </c>
-      <c r="G413" s="14" t="inlineStr">
-        <is>
-          <t>Rojo Esmerilado</t>
-        </is>
-      </c>
-      <c r="H413" s="15" t="inlineStr">
-        <is>
-          <t>$665.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="414" ht="16" customHeight="1">
-      <c r="A414" s="4" t="inlineStr"/>
-      <c r="B414" s="4" t="inlineStr"/>
-      <c r="C414" s="4" t="inlineStr"/>
-      <c r="D414" s="4" t="inlineStr"/>
-      <c r="E414" s="4" t="inlineStr"/>
-      <c r="F414" s="4" t="inlineStr">
-        <is>
-          <t>H.PBO35</t>
-        </is>
-      </c>
-      <c r="G414" s="4" t="inlineStr">
-        <is>
-          <t>Azul Esmerilado</t>
-        </is>
-      </c>
-      <c r="H414" s="5" t="inlineStr">
-        <is>
-          <t>$665.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="415" ht="16" customHeight="1">
-      <c r="A415" s="14" t="inlineStr"/>
-      <c r="B415" s="14" t="inlineStr"/>
-      <c r="C415" s="14" t="inlineStr"/>
-      <c r="D415" s="14" t="inlineStr"/>
-      <c r="E415" s="14" t="inlineStr"/>
-      <c r="F415" s="14" t="inlineStr">
-        <is>
-          <t>H.PBO37</t>
-        </is>
-      </c>
-      <c r="G415" s="14" t="inlineStr">
-        <is>
-          <t>Dorado</t>
-        </is>
-      </c>
-      <c r="H415" s="15" t="inlineStr">
-        <is>
-          <t>$794.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="416" ht="16" customHeight="1">
-      <c r="A416" s="14" t="inlineStr">
-        <is>
-          <t>Complementos</t>
-        </is>
-      </c>
-      <c r="B416" s="14" t="inlineStr">
-        <is>
-          <t>Filippo</t>
-        </is>
-      </c>
-      <c r="C416" s="14" t="inlineStr">
-        <is>
-          <t>Soportaborellas</t>
-        </is>
-      </c>
-      <c r="D416" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E416" s="14" t="inlineStr">
-        <is>
-          <t>Acrílico</t>
-        </is>
-      </c>
-      <c r="F416" s="14" t="inlineStr">
-        <is>
-          <t>H.PBO24</t>
-        </is>
-      </c>
-      <c r="G416" s="14" t="inlineStr">
-        <is>
-          <t>Transparente</t>
-        </is>
-      </c>
-      <c r="H416" s="15" t="inlineStr">
-        <is>
-          <t>$414.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="417" ht="16" customHeight="1">
-      <c r="A417" s="4" t="inlineStr"/>
-      <c r="B417" s="4" t="inlineStr"/>
-      <c r="C417" s="4" t="inlineStr"/>
-      <c r="D417" s="4" t="inlineStr"/>
-      <c r="E417" s="4" t="inlineStr"/>
-      <c r="F417" s="4" t="inlineStr">
-        <is>
-          <t>H.PBO26</t>
-        </is>
-      </c>
-      <c r="G417" s="4" t="inlineStr">
-        <is>
-          <t>Rojo</t>
-        </is>
-      </c>
-      <c r="H417" s="5" t="inlineStr">
-        <is>
-          <t>$414.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="418" ht="16" customHeight="1">
-      <c r="A418" s="14" t="inlineStr"/>
-      <c r="B418" s="14" t="inlineStr"/>
-      <c r="C418" s="14" t="inlineStr"/>
-      <c r="D418" s="14" t="inlineStr"/>
-      <c r="E418" s="14" t="inlineStr"/>
-      <c r="F418" s="14" t="inlineStr">
-        <is>
-          <t>H.PBO30</t>
-        </is>
-      </c>
-      <c r="G418" s="14" t="inlineStr">
-        <is>
-          <t>Turquesa</t>
-        </is>
-      </c>
-      <c r="H418" s="15" t="inlineStr">
-        <is>
-          <t>$414.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="419" ht="16" customHeight="1">
-      <c r="A419" s="14" t="inlineStr">
-        <is>
-          <t>Complementos</t>
-        </is>
-      </c>
-      <c r="B419" s="14" t="inlineStr">
-        <is>
-          <t>Bonnie &amp; Clyde</t>
-        </is>
-      </c>
-      <c r="C419" s="14" t="inlineStr">
-        <is>
-          <t>Sal y Pimienta</t>
-        </is>
-      </c>
-      <c r="D419" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E419" s="14" t="inlineStr">
-        <is>
-          <t>Acrílico</t>
-        </is>
-      </c>
-      <c r="F419" s="14" t="inlineStr">
-        <is>
-          <t>H.SAL.BEC1</t>
-        </is>
-      </c>
-      <c r="G419" s="14" t="inlineStr">
-        <is>
-          <t>Verde</t>
-        </is>
-      </c>
-      <c r="H419" s="15" t="inlineStr">
-        <is>
-          <t>$222.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="420" ht="16" customHeight="1">
-      <c r="A420" s="4" t="inlineStr"/>
-      <c r="B420" s="4" t="inlineStr"/>
-      <c r="C420" s="4" t="inlineStr"/>
-      <c r="D420" s="4" t="inlineStr"/>
-      <c r="E420" s="4" t="inlineStr"/>
-      <c r="F420" s="4" t="inlineStr">
-        <is>
-          <t>H.SAL.BEC2</t>
-        </is>
-      </c>
-      <c r="G420" s="4" t="inlineStr">
-        <is>
-          <t>Transparente</t>
-        </is>
-      </c>
-      <c r="H420" s="5" t="inlineStr">
-        <is>
-          <t>$222.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="421" ht="16" customHeight="1">
-      <c r="A421" s="14" t="inlineStr"/>
-      <c r="B421" s="14" t="inlineStr"/>
-      <c r="C421" s="14" t="inlineStr"/>
-      <c r="D421" s="14" t="inlineStr"/>
-      <c r="E421" s="14" t="inlineStr"/>
-      <c r="F421" s="14" t="inlineStr">
-        <is>
-          <t>H.SAL.BEC3</t>
-        </is>
-      </c>
-      <c r="G421" s="14" t="inlineStr">
-        <is>
-          <t>Azul</t>
-        </is>
-      </c>
-      <c r="H421" s="15" t="inlineStr">
-        <is>
-          <t>$222.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="422" ht="16" customHeight="1">
-      <c r="A422" s="4" t="inlineStr"/>
-      <c r="B422" s="4" t="inlineStr"/>
-      <c r="C422" s="4" t="inlineStr"/>
-      <c r="D422" s="4" t="inlineStr"/>
-      <c r="E422" s="4" t="inlineStr"/>
-      <c r="F422" s="4" t="inlineStr">
-        <is>
-          <t>H.SAL.BEC5</t>
-        </is>
-      </c>
-      <c r="G422" s="4" t="inlineStr">
-        <is>
-          <t>Rojo</t>
-        </is>
-      </c>
-      <c r="H422" s="5" t="inlineStr">
-        <is>
-          <t>$222.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="423" ht="16" customHeight="1">
-      <c r="A423" s="14" t="inlineStr"/>
-      <c r="B423" s="14" t="inlineStr"/>
-      <c r="C423" s="14" t="inlineStr"/>
-      <c r="D423" s="14" t="inlineStr"/>
-      <c r="E423" s="14" t="inlineStr"/>
-      <c r="F423" s="14" t="inlineStr">
-        <is>
-          <t>H.SAL.BEC6</t>
-        </is>
-      </c>
-      <c r="G423" s="14" t="inlineStr">
-        <is>
-          <t>Dorado</t>
-        </is>
-      </c>
-      <c r="H423" s="15" t="inlineStr">
-        <is>
-          <t>$222.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="424" ht="16" customHeight="1">
-      <c r="A424" s="14" t="inlineStr">
-        <is>
-          <t>Complementos</t>
-        </is>
-      </c>
-      <c r="B424" s="14" t="inlineStr">
-        <is>
-          <t>Casanova</t>
-        </is>
-      </c>
-      <c r="C424" s="14" t="inlineStr">
-        <is>
-          <t>Salero</t>
-        </is>
-      </c>
-      <c r="D424" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E424" s="14" t="inlineStr">
-        <is>
-          <t>Acrílico</t>
-        </is>
-      </c>
-      <c r="F424" s="14" t="inlineStr">
-        <is>
-          <t>H.SAL.CAS1</t>
-        </is>
-      </c>
-      <c r="G424" s="14" t="inlineStr">
-        <is>
-          <t>Transparente</t>
-        </is>
-      </c>
-      <c r="H424" s="15" t="inlineStr">
-        <is>
-          <t>$55.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="425" ht="16" customHeight="1">
-      <c r="A425" s="4" t="inlineStr"/>
-      <c r="B425" s="4" t="inlineStr"/>
-      <c r="C425" s="4" t="inlineStr"/>
-      <c r="D425" s="4" t="inlineStr"/>
-      <c r="E425" s="4" t="inlineStr"/>
-      <c r="F425" s="4" t="inlineStr">
-        <is>
-          <t>H.SAL.CAS2</t>
-        </is>
-      </c>
-      <c r="G425" s="4" t="inlineStr">
-        <is>
-          <t>Ahumado</t>
-        </is>
-      </c>
-      <c r="H425" s="5" t="inlineStr">
-        <is>
-          <t>$55.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="426" ht="16" customHeight="1">
-      <c r="A426" s="14" t="inlineStr"/>
-      <c r="B426" s="14" t="inlineStr"/>
-      <c r="C426" s="14" t="inlineStr"/>
-      <c r="D426" s="14" t="inlineStr"/>
-      <c r="E426" s="14" t="inlineStr"/>
-      <c r="F426" s="14" t="inlineStr">
-        <is>
-          <t>H.SAL.CAS3</t>
-        </is>
-      </c>
-      <c r="G426" s="14" t="inlineStr">
-        <is>
-          <t>Verde</t>
-        </is>
-      </c>
-      <c r="H426" s="15" t="inlineStr">
-        <is>
-          <t>$55.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="427" ht="16" customHeight="1">
-      <c r="A427" s="4" t="inlineStr"/>
-      <c r="B427" s="4" t="inlineStr"/>
-      <c r="C427" s="4" t="inlineStr"/>
-      <c r="D427" s="4" t="inlineStr"/>
-      <c r="E427" s="4" t="inlineStr"/>
-      <c r="F427" s="4" t="inlineStr">
-        <is>
-          <t>H.SAL.CAS4</t>
-        </is>
-      </c>
-      <c r="G427" s="4" t="inlineStr">
-        <is>
-          <t>Rojo</t>
-        </is>
-      </c>
-      <c r="H427" s="5" t="inlineStr">
-        <is>
-          <t>$55.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="428" ht="16" customHeight="1">
-      <c r="A428" s="14" t="inlineStr">
-        <is>
-          <t>Complementos</t>
-        </is>
-      </c>
-      <c r="B428" s="14" t="inlineStr">
-        <is>
-          <t>Caterina &amp; Vittoria</t>
-        </is>
-      </c>
-      <c r="C428" s="14" t="inlineStr">
-        <is>
-          <t>Sal y Pimienta</t>
-        </is>
-      </c>
-      <c r="D428" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E428" s="14" t="inlineStr">
-        <is>
-          <t>Acrílico</t>
-        </is>
-      </c>
-      <c r="F428" s="14" t="inlineStr">
-        <is>
-          <t>H.SAL.CEV1</t>
-        </is>
-      </c>
-      <c r="G428" s="14" t="inlineStr">
-        <is>
-          <t>Transparente</t>
-        </is>
-      </c>
-      <c r="H428" s="15" t="inlineStr">
+      <c r="H403" s="5" t="inlineStr">
         <is>
           <t>$269.000</t>
         </is>
       </c>
     </row>
-    <row r="429" ht="16" customHeight="1">
-      <c r="A429" s="4" t="inlineStr"/>
-      <c r="B429" s="4" t="inlineStr"/>
-      <c r="C429" s="4" t="inlineStr"/>
-      <c r="D429" s="4" t="inlineStr"/>
-      <c r="E429" s="4" t="inlineStr"/>
-      <c r="F429" s="4" t="inlineStr">
-        <is>
-          <t>H.SAL.CEV2</t>
-        </is>
-      </c>
-      <c r="G429" s="4" t="inlineStr">
-        <is>
-          <t>Rubí</t>
-        </is>
-      </c>
-      <c r="H429" s="5" t="inlineStr">
-        <is>
-          <t>$269.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="430" ht="16" customHeight="1">
-      <c r="A430" s="14" t="inlineStr"/>
-      <c r="B430" s="14" t="inlineStr"/>
-      <c r="C430" s="14" t="inlineStr"/>
-      <c r="D430" s="14" t="inlineStr"/>
-      <c r="E430" s="14" t="inlineStr"/>
-      <c r="F430" s="14" t="inlineStr">
-        <is>
-          <t>H.SAL.CEV3</t>
-        </is>
-      </c>
-      <c r="G430" s="14" t="inlineStr">
-        <is>
-          <t>Azul</t>
-        </is>
-      </c>
-      <c r="H430" s="15" t="inlineStr">
-        <is>
-          <t>$269.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="431" ht="16" customHeight="1">
-      <c r="A431" s="4" t="inlineStr"/>
-      <c r="B431" s="4" t="inlineStr"/>
-      <c r="C431" s="4" t="inlineStr"/>
-      <c r="D431" s="4" t="inlineStr"/>
-      <c r="E431" s="4" t="inlineStr"/>
-      <c r="F431" s="4" t="inlineStr">
-        <is>
-          <t>H.SAL.CEV4</t>
-        </is>
-      </c>
-      <c r="G431" s="4" t="inlineStr">
-        <is>
-          <t>Verde</t>
-        </is>
-      </c>
-      <c r="H431" s="5" t="inlineStr">
-        <is>
-          <t>$269.000</t>
-        </is>
-      </c>
-    </row>
+    <row r="404" ht="16" customHeight="1"/>
+    <row r="405" ht="16" customHeight="1"/>
+    <row r="406" ht="16" customHeight="1"/>
+    <row r="407" ht="16" customHeight="1"/>
+    <row r="408" ht="16" customHeight="1"/>
+    <row r="409" ht="16" customHeight="1"/>
+    <row r="410" ht="16" customHeight="1"/>
+    <row r="411" ht="16" customHeight="1"/>
+    <row r="412" ht="16" customHeight="1"/>
+    <row r="413" ht="16" customHeight="1"/>
+    <row r="414" ht="16" customHeight="1"/>
+    <row r="415" ht="16" customHeight="1"/>
+    <row r="416" ht="16" customHeight="1"/>
+    <row r="417" ht="16" customHeight="1"/>
+    <row r="418" ht="16" customHeight="1"/>
+    <row r="419" ht="16" customHeight="1"/>
+    <row r="420" ht="16" customHeight="1"/>
+    <row r="421" ht="16" customHeight="1"/>
+    <row r="422" ht="16" customHeight="1"/>
+    <row r="423" ht="16" customHeight="1"/>
+    <row r="424" ht="16" customHeight="1"/>
+    <row r="425" ht="16" customHeight="1"/>
+    <row r="426" ht="16" customHeight="1"/>
+    <row r="427" ht="16" customHeight="1"/>
+    <row r="428" ht="16" customHeight="1"/>
+    <row r="429" ht="16" customHeight="1"/>
+    <row r="430" ht="16" customHeight="1"/>
+    <row r="431" ht="16" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11891,92 +11123,92 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Copas y Vasos</t>
+          <t>Alzadas</t>
         </is>
       </c>
       <c r="B2" s="17" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="C2" s="17" t="n">
-        <v>171</v>
+        <v>12</v>
       </c>
       <c r="D2" s="17" t="inlineStr">
         <is>
-          <t>$67.000</t>
+          <t>$177.000</t>
         </is>
       </c>
       <c r="E2" s="17" t="inlineStr">
         <is>
-          <t>$170.000</t>
+          <t>$672.000</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="18" t="inlineStr">
         <is>
-          <t>Alzadas</t>
+          <t>Complementos</t>
         </is>
       </c>
       <c r="B3" s="19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" s="19" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D3" s="19" t="inlineStr">
         <is>
-          <t>$177.000</t>
+          <t>$55.000</t>
         </is>
       </c>
       <c r="E3" s="19" t="inlineStr">
         <is>
-          <t>$672.000</t>
+          <t>$794.000</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="20" t="inlineStr">
         <is>
-          <t>Ensaladeras</t>
+          <t>Copas y Vasos</t>
         </is>
       </c>
       <c r="B4" s="21" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="C4" s="21" t="n">
-        <v>20</v>
+        <v>171</v>
       </c>
       <c r="D4" s="21" t="inlineStr">
         <is>
-          <t>$118.000</t>
+          <t>$67.000</t>
         </is>
       </c>
       <c r="E4" s="21" t="inlineStr">
         <is>
-          <t>$621.000</t>
+          <t>$170.000</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="22" t="inlineStr">
         <is>
-          <t>Platos</t>
+          <t>Ensaladeras</t>
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="C5" s="23" t="n">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="D5" s="23" t="inlineStr">
         <is>
-          <t>$124.000</t>
+          <t>$118.000</t>
         </is>
       </c>
       <c r="E5" s="23" t="inlineStr">
         <is>
-          <t>$550.000</t>
+          <t>$621.000</t>
         </is>
       </c>
     </row>
@@ -12006,23 +11238,23 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>Complementos</t>
+          <t>Platos</t>
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
-          <t>$55.000</t>
+          <t>$124.000</t>
         </is>
       </c>
       <c r="E7" s="27" t="inlineStr">
         <is>
-          <t>$1.459.000</t>
+          <t>$550.000</t>
         </is>
       </c>
     </row>
@@ -12033,10 +11265,10 @@
         </is>
       </c>
       <c r="B8" s="29" t="n">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="C8" s="29" t="n">
-        <v>430</v>
+        <v>402</v>
       </c>
       <c r="D8" s="30" t="n"/>
       <c r="E8" s="30" t="n"/>

</xml_diff>